<commit_message>
remove the literal word actuator to avoid data contamination
</commit_message>
<xml_diff>
--- a/data/actuator_examples.xlsx
+++ b/data/actuator_examples.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\scripts\hil\hil-test-case-gen\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A4A61B-4DFB-474E-9067-F3CBE51942A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A16E12D8-0035-4CBB-9D23-A1C5A978B49C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{4E185E56-D21A-4CEB-9BC3-DCDD147047F3}"/>
   </bookViews>
@@ -38,22 +38,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>In case of actuator overheating, the EPS system shall reduce power to the actuator and alert the driver.</t>
+    <t>Requirement</t>
   </si>
   <si>
-    <t>Faults in the engine actuator that result in loss of power shall trigger the system to activate hazard lights and alert nearby vehicles.</t>
+    <t>In case of overheating, the EPS system shall reduce power to the and alert the driver.</t>
   </si>
   <si>
-    <t>The system must guide the vehicle to the nearest safe stop zone in the event of a comprehensive actuator failure impacting multiple systems.</t>
+    <t>Faults in the engine that result in loss of power shall trigger the system to activate hazard lights and alert nearby vehicles.</t>
   </si>
   <si>
-    <t>Automatic actuator realignment and calibration procedures should execute after fault detection to confirm integrity before reactivation.</t>
+    <t>The system must guide the vehicle to the nearest safe stop zone in the event of a comprehensive failure impacting multiple systems.</t>
   </si>
   <si>
-    <t>The steering system shall limit the actuator's maximum force output if excessive torque is detected to prevent mechanical damage.</t>
+    <t>Automatic realignment and calibration procedures should execute after fault detection to confirm integrity before reactivation.</t>
   </si>
   <si>
-    <t>Requirement</t>
+    <t>The steering system shall limit the maximum force output if excessive torque is detected to prevent mechanical damage.</t>
   </si>
 </sst>
 </file>
@@ -118,9 +118,6 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -158,6 +155,9 @@
       </font>
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -172,10 +172,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73751A98-C4FC-40B7-94D7-6F01BDD0DAFC}" name="Table1" displayName="Table1" ref="A1:A6" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73751A98-C4FC-40B7-94D7-6F01BDD0DAFC}" name="Table1" displayName="Table1" ref="A1:A6" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
   <autoFilter ref="A1:A6" xr:uid="{73751A98-C4FC-40B7-94D7-6F01BDD0DAFC}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{9D4BE916-78CC-42EA-A7E0-82E0B310E701}" name="Requirement" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{9D4BE916-78CC-42EA-A7E0-82E0B310E701}" name="Requirement" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -506,32 +506,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="15.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.55000000000000004">

</xml_diff>